<commit_message>
atualizacao de sexta feira
</commit_message>
<xml_diff>
--- a/data/cepea-consulta-açucar-cristal.reparado.xlsx
+++ b/data/cepea-consulta-açucar-cristal.reparado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filipe.guidastri\Documents\Projetos\acompanhamento-cotacao\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4ABF75E0-8803-4346-B522-F224A963552C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE7EAD10-F7C2-4818-9389-13F9445239E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5760" yWindow="3396" windowWidth="17280" windowHeight="8964"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="1115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1256" uniqueCount="1117">
   <si>
     <t>Açúcar | INDICADOR DO AÇÚCAR CRISTAL BRANCO CEPEA/ESALQ - SÃO PAULO</t>
   </si>
@@ -3376,6 +3376,12 @@
   </si>
   <si>
     <t>21,74</t>
+  </si>
+  <si>
+    <t>28/08/2025</t>
+  </si>
+  <si>
+    <t>118,60</t>
   </si>
 </sst>
 </file>
@@ -3827,7 +3833,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J419"/>
+  <dimension ref="A1:J420"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.88671875" customWidth="1"/>
@@ -8455,6 +8461,17 @@
       </c>
       <c r="C419" s="3" t="s">
         <v>1114</v>
+      </c>
+    </row>
+    <row r="420" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A420" s="3" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B420" s="3" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C420" s="3" t="s">
+        <v>1103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>